<commit_message>
update telemetry csv file
</commit_message>
<xml_diff>
--- a/Iracing/Data_Logs/stint_telemetry_summary.xlsx
+++ b/Iracing/Data_Logs/stint_telemetry_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,6 +628,174 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>92.953</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>13:24:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" t="n">
+        <v>82.827</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>13:26:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>83.55500000000001</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>13:27:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" t="n">
+        <v>82.947</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>13:29:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" t="n">
+        <v>82.498</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="E13" t="n">
+        <v>9</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>13:30:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="E14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>13:31:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tomaz Nunes</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>81.812</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>13:33:09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>